<commit_message>
Ticketing, messages , auditability, Mock fintech tools, RAG and provider layer, LangGraph backend workflow
</commit_message>
<xml_diff>
--- a/data/seed/master_excel/samadhan_demo_seed_data.xlsx
+++ b/data/seed/master_excel/samadhan_demo_seed_data.xlsx
@@ -1494,7 +1494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1601,6 +1601,866 @@
       <c r="U1" t="inlineStr">
         <is>
           <t>closed_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TKT-2026-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USR-CUST-001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SES-2026-0001</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>tier_2_conversation</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>loan_application_status</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>auto_resolved</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Loan pending due to KYC</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Customer asked why loan application is still pending.</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>My loan is still pending. What is the issue?</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Your application is pending KYC document verification.</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TKT-2026-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CUST-002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USR-CUST-002</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SES-2026-0002</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>tier_2_conversation</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>rejection_reason</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>auto_closed</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Loan rejection explanation</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Customer requested rejection reason for declined application.</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Why was my loan rejected?</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Your application did not meet current eligibility criteria.</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Customer received safe rejection explanation.</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TKT-2026-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CUST-003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USR-CUST-003</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SES-2026-0003</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>human_review</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>emi_payment_issue</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>escalated_to_human</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Duplicate EMI debit</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Customer reported EMI was deducted twice for the same cycle.</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>My EMI was deducted twice this month.</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Your case has been escalated for human review.</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Financial dispute — duplicate EMI debit requires human review.</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TKT-2026-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CUST-004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USR-CUST-004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SES-2026-0004</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>tier_1_service_request</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>noc_closure_certificate</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>NOC pending after loan closure</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Customer closed loan and is waiting for NOC document.</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>I closed my loan. Where is my NOC?</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>We will create a service request for your NOC.</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TKT-2026-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CUST-005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USR-CUST-005</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SES-2026-0005</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>human_review</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>bureau_reporting_issue</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>under_review</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>CIBIL still shows active loan</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Customer reports bureau still shows closed loan as active.</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>CIBIL still shows my loan as active after closure.</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>A support agent is reviewing your bureau reporting case.</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>USR-AGENT-001</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Bureau/CIBIL mismatch requires human review.</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TKT-2026-0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>CUST-006</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USR-CUST-006</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SES-2026-0006</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>human_review</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>fraud_security_issue</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>critical</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>escalated_to_human</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Unauthorized transaction SMS alert</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Customer received SMS for a transaction they did not make.</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>I got an SMS for a transaction I did not make.</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Your security concern has been escalated immediately.</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Fraud/security alert — mandatory human review.</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TKT-2026-0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CUST-007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USR-CUST-007</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SES-2026-0007</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>tier_2_conversation</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>topup_offer</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>auto_resolved</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Top-up eligibility inquiry</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Customer asked about pre-approved top-up offer eligibility.</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Am I eligible for a top-up loan?</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>You have a pre-approved top-up offer available.</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TKT-2026-0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CUST-008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>USR-CUST-008</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SES-2026-0008</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>tier_2_conversation</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>topup_offer</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>auto_closed</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Top-up not eligible</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Customer asked about top-up but is not eligible.</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Can I get a top-up on my loan?</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>No pre-approved top-up offer is available at this time.</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Customer received eligibility explanation.</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TKT-2026-0009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CUST-009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>USR-CUST-009</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SES-2026-0009</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>tier_1_service_request</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>rm_redirection</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>RM callback request</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Customer wants to speak with relationship manager.</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>I want to speak to my RM.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>We will register a callback request for your RM.</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TKT-2026-0010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CUST-010</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>USR-CUST-010</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SES-2026-0010</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>tier_1_service_request</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>loan_statement_request</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Loan statement for tax filing</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Customer needs loan statement document.</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>web_chat</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Please generate my loan statement for tax filing.</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>We will create a loan statement service request.</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
         </is>
       </c>
     </row>
@@ -1615,7 +2475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1662,6 +2522,896 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>created_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MSG-2026-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TKT-2026-0001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SES-2026-0001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>My loan is still pending. What is the issue?</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>USR-CUST-001</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MSG-2026-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TKT-2026-0001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SES-2026-0001</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CUST-001</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Your application is pending KYC document verification.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MSG-2026-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TKT-2026-0002</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>SES-2026-0002</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CUST-002</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Why was my loan rejected?</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>USR-CUST-002</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MSG-2026-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TKT-2026-0002</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SES-2026-0002</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CUST-002</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Your application did not meet current eligibility criteria.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MSG-2026-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TKT-2026-0003</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SES-2026-0003</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CUST-003</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>My EMI was deducted twice this month.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>USR-CUST-003</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MSG-2026-0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TKT-2026-0003</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SES-2026-0003</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CUST-003</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Your case has been escalated for human review.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MSG-2026-0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TKT-2026-0004</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SES-2026-0004</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>CUST-004</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>I closed my loan. Where is my NOC?</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>USR-CUST-004</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MSG-2026-0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TKT-2026-0004</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SES-2026-0004</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CUST-004</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>We will create a service request for your NOC.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MSG-2026-0009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TKT-2026-0005</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SES-2026-0005</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CUST-005</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>CIBIL still shows my loan as active after closure.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>USR-CUST-005</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MSG-2026-0010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TKT-2026-0005</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SES-2026-0005</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CUST-005</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>A support agent is reviewing your bureau reporting case.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MSG-2026-0011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TKT-2026-0006</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SES-2026-0006</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CUST-006</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>I got an SMS for a transaction I did not make.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>USR-CUST-006</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MSG-2026-0012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TKT-2026-0006</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SES-2026-0006</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CUST-006</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Your security concern has been escalated immediately.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MSG-2026-0013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TKT-2026-0007</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SES-2026-0007</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CUST-007</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Am I eligible for a top-up loan?</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>USR-CUST-007</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>MSG-2026-0014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TKT-2026-0007</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SES-2026-0007</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CUST-007</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>You have a pre-approved top-up offer available.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MSG-2026-0015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TKT-2026-0008</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SES-2026-0008</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CUST-008</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Can I get a top-up on my loan?</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>USR-CUST-008</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MSG-2026-0016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TKT-2026-0008</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>SES-2026-0008</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CUST-008</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>No pre-approved top-up offer is available at this time.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>MSG-2026-0017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TKT-2026-0009</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SES-2026-0009</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CUST-009</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>I want to speak to my RM.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>USR-CUST-009</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>MSG-2026-0018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TKT-2026-0009</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SES-2026-0009</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CUST-009</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>We will register a callback request for your RM.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MSG-2026-0019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TKT-2026-0010</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SES-2026-0010</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CUST-010</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Please generate my loan statement for tax filing.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>USR-CUST-010</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MSG-2026-0020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TKT-2026-0010</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SES-2026-0010</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>CUST-010</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>We will create a loan statement service request.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>{"source": "seed"}</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-06-13T12:00:00+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>